<commit_message>
feat: expand district demo and paper-to-Excel workflow
Add twenty basemap-aligned synthetic locations, richer outreach histories, and a reviewed Excel merge/export workflow. Refine district framing, automatic floor expansion, camera rotation, and foreground visibility.

Validate with 60 tests, TypeScript, ESLint, production build, and browser workflow checks.
</commit_message>
<xml_diff>
--- a/public/demo/careflow-field-outreach-demo.xlsx
+++ b/public/demo/careflow-field-outreach-demo.xlsx
@@ -430,7 +430,7 @@
         <v>notice</v>
       </c>
       <c r="B3" t="str">
-        <v>所有業務資料、姓名、座標、地址與樓層單位結構均為合成示例，並非真實住戶或已核實資料。</v>
+        <v>業務資料、姓名、地址與樓層單位結構均為合成示例；占地輪廓參照 OpenStreetMap 底圖，不表示真實大廈身份或住戶資料已核實。</v>
       </c>
     </row>
   </sheetData>
@@ -1910,7 +1910,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1929,12 +1929,15 @@
         <v>lat</v>
       </c>
       <c r="F1" t="str">
+        <v>footprint</v>
+      </c>
+      <c r="G1" t="str">
         <v>floorCount</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>layoutDeclared</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>initialCoverage</v>
       </c>
     </row>
@@ -1949,18 +1952,21 @@
         <v>西營盤示範街 1 號（合成）</v>
       </c>
       <c r="D2">
-        <v>114.1418</v>
+        <v>114.14178818464279</v>
       </c>
       <c r="E2">
-        <v>22.2863</v>
-      </c>
-      <c r="F2">
+        <v>22.286363930711317</v>
+      </c>
+      <c r="F2" t="str">
+        <v>[[114.14168894290924,22.286500432351488],[114.1418981552124,22.286495468660235],[114.14189279079437,22.286227429071147],[114.14167821407318,22.286237356472498],[114.14168894290924,22.286500432351488]]</v>
+      </c>
+      <c r="G2">
         <v>8</v>
       </c>
-      <c r="G2" t="b">
+      <c r="H2" t="b">
         <v>1</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>UNVISITED</v>
       </c>
     </row>
@@ -1975,18 +1981,21 @@
         <v>西營盤示範街 8 號（合成）</v>
       </c>
       <c r="D3">
-        <v>114.14252</v>
+        <v>114.14255797863007</v>
       </c>
       <c r="E3">
-        <v>22.28652</v>
-      </c>
-      <c r="F3">
+        <v>22.28661211534631</v>
+      </c>
+      <c r="F3" t="str">
+        <v>[[114.14262235164642,22.286664234063778],[114.14262235164642,22.286619560888553],[114.14259016513824,22.286624524575387],[114.14258480072021,22.286589778763798],[114.14263308048248,22.286589778763798],[114.14263308048248,22.286555032943582],[114.14248287677765,22.286559996632704],[114.14248287677765,22.28659474245171],[114.14253115653992,22.28659474245171],[114.14253115653992,22.286624524575387],[114.14249897003174,22.286624524575387],[114.14249897003174,22.286669197749035],[114.14262235164642,22.286664234063778]]</v>
+      </c>
+      <c r="G3">
         <v>2</v>
       </c>
-      <c r="G3" t="b">
+      <c r="H3" t="b">
         <v>1</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>UNVISITED</v>
       </c>
     </row>
@@ -2001,18 +2010,21 @@
         <v>西營盤示範街 16 號（合成）</v>
       </c>
       <c r="D4">
-        <v>114.14135</v>
+        <v>114.14136976003647</v>
       </c>
       <c r="E4">
-        <v>22.28681</v>
+        <v>22.286808180844794</v>
       </c>
       <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="b">
+        <v>[[114.1414475440979,22.286733725641312],[114.14129197597504,22.286733725641312],[114.14129197597504,22.286882636048276],[114.1414475440979,22.286877672370593],[114.1414475440979,22.286733725641312]]</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="b">
         <v>0</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>UNKNOWN</v>
       </c>
     </row>
@@ -2027,24 +2039,27 @@
         <v>西營盤示範街 24 號（合成）</v>
       </c>
       <c r="D5">
-        <v>114.14211</v>
+        <v>114.14208590984344</v>
       </c>
       <c r="E5">
-        <v>22.28582</v>
+        <v>22.28576580411479</v>
       </c>
       <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="b">
+        <v>[[114.14213418960571,22.285825368723906],[114.14212882518768,22.28570127579063],[114.14203763008118,22.285706239510063],[114.1420429944992,22.285830332438948],[114.14213418960571,22.285825368723906]]</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="b">
         <v>0</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>UNKNOWN</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>